<commit_message>
docs: hoan thien ho so BT1 va khai bao AI
Cap nhat API contract theo track SE, bo sung validation va truy vet User Story; dieu chinh so do Use Case va kien truc; cap nhat tai lieu Word, Excel va noi dung khai bao su dung AI; xac nhan smoke test thanh cong.
</commit_message>
<xml_diff>
--- a/docs/ai-disclosure.xlsx
+++ b/docs/ai-disclosure.xlsx
@@ -1,58 +1,79 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\bài tập chuyen đề tn1\docs\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D20EF9A-E657-4AF9-9B5E-AE8065820343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Khai bao AI" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+  <si>
+    <t>Công cụ đã sử dụng</t>
+  </si>
+  <si>
+    <t>Phần sản phẩm có sử dụng AI hỗ trợ</t>
+  </si>
+  <si>
+    <t>GitHub Copilot/Copilot Chat: đọc và tóm tắt case study, gợi ý phạm vi L2, tạo mã khung Node.js/Express, viết smoke test và hỗ trợ kiểm tra tài liệu.</t>
+  </si>
+  <si>
+    <t>Phiếu phạm vi buổi 2 và danh sách User Story cho luồng L2; mã khung endpoint GET /health; smoke test trong tests/smoke-test.js.</t>
+  </si>
+  <si>
+    <t>ChatGPT: hỗ trợ diễn đạt User Story, hướng dẫn cấu trúc repo, .gitignore, .env.example, README và cách sử dụng dữ liệu mẫu.</t>
+  </si>
+  <si>
+    <t>Cấu trúc thư mục repo, file cấu hình ban đầu, README, hướng dẫn dữ liệu L2, tài liệu cấu hình môi trường và mẫu dữ liệu nhỏ trong data/sample/.</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -60,18 +81,49 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+  <cellXfs count="3">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Accent1" xfId="1" builtinId="29"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,40 +448,42 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="75.83203125" customWidth="1"/>
-    <col min="2" max="2" width="85.83203125" customWidth="1"/>
+    <col min="1" max="1" width="75.77734375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="85.77734375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Công cụ đã sử dụng</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Phần sản phẩm có sử dụng AI hỗ trợ</v>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>GitHub Copilot/Copilot Chat: đọc và tóm tắt case study, gợi ý phạm vi L2, tạo mã khung Node.js/Express, viết smoke test và hỗ trợ kiểm tra tài liệu.</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Phiếu phạm vi buổi 2 và danh sách User Story cho luồng L2; mã khung endpoint GET /health; smoke test trong tests/smoke-test.js.</v>
+    <row r="2" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>ChatGPT: hỗ trợ diễn đạt User Story, hướng dẫn cấu trúc repo, .gitignore, .env.example, README và cách sử dụng dữ liệu mẫu.</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Cấu trúc thư mục repo, file cấu hình ban đầu, README, hướng dẫn dữ liệu L2, tài liệu cấu hình môi trường và mẫu dữ liệu nhỏ trong data/sample/.</v>
+    <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B3"/>
+    <ignoredError sqref="A1:B3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>